<commit_message>
add printing ability for pre and post form
</commit_message>
<xml_diff>
--- a/travel-manager/FY26_ISTE_Travel_Form_Template.xlsx
+++ b/travel-manager/FY26_ISTE_Travel_Form_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nmgov-my.sharepoint.com/personal/cole_sullivan_hca_nm_gov/Documents/Desktop/practice code/monday-test-app/travel-manager/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="87" documentId="13_ncr:1_{31D518EC-BF6C-4982-87C1-3797D64F72E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{425F23BE-0668-42BC-A10D-31F456BA6E79}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="13_ncr:1_{31D518EC-BF6C-4982-87C1-3797D64F72E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4B63094-C0CC-496B-9C96-3D1EA32FD889}"/>
   <bookViews>
-    <workbookView xWindow="3795" yWindow="2055" windowWidth="25755" windowHeight="16470" xr2:uid="{829E26D7-8683-4007-91D0-8026F11B546D}"/>
+    <workbookView xWindow="4050" yWindow="1590" windowWidth="25755" windowHeight="16470" xr2:uid="{829E26D7-8683-4007-91D0-8026F11B546D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1137,6 +1137,194 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="46" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="46" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="3" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="3" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="3" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="3" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="4" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="5" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="4" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="4" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1146,6 +1334,74 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1168,13 +1424,218 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1183,10 +1644,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1194,21 +1651,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1263,14 +1709,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1304,467 +1742,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="3" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="3" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="4" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="4" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="4" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="3" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="3" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="5" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="46" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="46" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1994,6 +1994,10 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3774,428 +3778,428 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="207" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="73" t="s">
+      <c r="B1" s="208"/>
+      <c r="C1" s="208"/>
+      <c r="D1" s="208"/>
+      <c r="E1" s="208"/>
+      <c r="F1" s="208"/>
+      <c r="G1" s="209"/>
+      <c r="H1" s="210" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="74"/>
-      <c r="J1" s="74"/>
-      <c r="K1" s="74"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="82" t="s">
+      <c r="I1" s="211"/>
+      <c r="J1" s="211"/>
+      <c r="K1" s="211"/>
+      <c r="L1" s="212"/>
+      <c r="M1" s="219" t="s">
         <v>2</v>
       </c>
-      <c r="N1" s="84">
+      <c r="N1" s="189">
         <v>1</v>
       </c>
-      <c r="O1" s="86"/>
-      <c r="P1" s="87"/>
-      <c r="Q1" s="87"/>
-      <c r="R1" s="87"/>
-      <c r="S1" s="87"/>
-      <c r="T1" s="88"/>
+      <c r="O1" s="221"/>
+      <c r="P1" s="222"/>
+      <c r="Q1" s="222"/>
+      <c r="R1" s="222"/>
+      <c r="S1" s="222"/>
+      <c r="T1" s="223"/>
     </row>
     <row r="2" spans="1:25" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="227" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="93"/>
-      <c r="C2" s="93"/>
-      <c r="D2" s="93"/>
-      <c r="E2" s="93"/>
-      <c r="F2" s="93"/>
-      <c r="G2" s="94"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="77"/>
-      <c r="J2" s="77"/>
-      <c r="K2" s="77"/>
-      <c r="L2" s="78"/>
-      <c r="M2" s="83"/>
-      <c r="N2" s="85"/>
-      <c r="O2" s="89"/>
-      <c r="P2" s="90"/>
-      <c r="Q2" s="90"/>
-      <c r="R2" s="90"/>
-      <c r="S2" s="90"/>
-      <c r="T2" s="91"/>
+      <c r="B2" s="228"/>
+      <c r="C2" s="228"/>
+      <c r="D2" s="228"/>
+      <c r="E2" s="228"/>
+      <c r="F2" s="228"/>
+      <c r="G2" s="229"/>
+      <c r="H2" s="213"/>
+      <c r="I2" s="214"/>
+      <c r="J2" s="214"/>
+      <c r="K2" s="214"/>
+      <c r="L2" s="215"/>
+      <c r="M2" s="220"/>
+      <c r="N2" s="60"/>
+      <c r="O2" s="224"/>
+      <c r="P2" s="225"/>
+      <c r="Q2" s="225"/>
+      <c r="R2" s="225"/>
+      <c r="S2" s="225"/>
+      <c r="T2" s="226"/>
     </row>
     <row r="3" spans="1:25" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="196" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="165" t="s">
         <v>61</v>
       </c>
-      <c r="C3" s="84"/>
-      <c r="D3" s="84"/>
-      <c r="E3" s="84"/>
-      <c r="F3" s="84"/>
-      <c r="G3" s="84"/>
-      <c r="H3" s="76"/>
-      <c r="I3" s="77"/>
-      <c r="J3" s="77"/>
-      <c r="K3" s="77"/>
-      <c r="L3" s="78"/>
-      <c r="M3" s="95" t="s">
+      <c r="C3" s="189"/>
+      <c r="D3" s="189"/>
+      <c r="E3" s="189"/>
+      <c r="F3" s="189"/>
+      <c r="G3" s="189"/>
+      <c r="H3" s="213"/>
+      <c r="I3" s="214"/>
+      <c r="J3" s="214"/>
+      <c r="K3" s="214"/>
+      <c r="L3" s="215"/>
+      <c r="M3" s="230" t="s">
         <v>4</v>
       </c>
-      <c r="N3" s="84">
+      <c r="N3" s="189">
         <v>63000</v>
       </c>
-      <c r="O3" s="55" t="s">
+      <c r="O3" s="134" t="s">
         <v>5</v>
       </c>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="59"/>
+      <c r="P3" s="165"/>
+      <c r="Q3" s="199"/>
+      <c r="R3" s="199"/>
+      <c r="S3" s="199"/>
+      <c r="T3" s="200"/>
     </row>
     <row r="4" spans="1:25" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="64"/>
-      <c r="B4" s="60"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
-      <c r="E4" s="85"/>
-      <c r="F4" s="85"/>
-      <c r="G4" s="85"/>
-      <c r="H4" s="79"/>
-      <c r="I4" s="80"/>
-      <c r="J4" s="80"/>
-      <c r="K4" s="80"/>
-      <c r="L4" s="81"/>
-      <c r="M4" s="96" t="s">
+      <c r="A4" s="203"/>
+      <c r="B4" s="191"/>
+      <c r="C4" s="60"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="60"/>
+      <c r="G4" s="60"/>
+      <c r="H4" s="216"/>
+      <c r="I4" s="217"/>
+      <c r="J4" s="217"/>
+      <c r="K4" s="217"/>
+      <c r="L4" s="218"/>
+      <c r="M4" s="231" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="85"/>
-      <c r="O4" s="56" t="s">
+      <c r="N4" s="60"/>
+      <c r="O4" s="198" t="s">
         <v>7</v>
       </c>
-      <c r="P4" s="60"/>
-      <c r="Q4" s="61"/>
-      <c r="R4" s="61"/>
-      <c r="S4" s="61"/>
-      <c r="T4" s="62"/>
+      <c r="P4" s="191"/>
+      <c r="Q4" s="201"/>
+      <c r="R4" s="201"/>
+      <c r="S4" s="201"/>
+      <c r="T4" s="202"/>
     </row>
     <row r="5" spans="1:25" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="196" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="57"/>
-      <c r="C5" s="65"/>
-      <c r="D5" s="65"/>
-      <c r="E5" s="65"/>
-      <c r="F5" s="66"/>
-      <c r="G5" s="97" t="s">
+      <c r="B5" s="165"/>
+      <c r="C5" s="166"/>
+      <c r="D5" s="166"/>
+      <c r="E5" s="166"/>
+      <c r="F5" s="167"/>
+      <c r="G5" s="193" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="98"/>
-      <c r="I5" s="99" t="s">
+      <c r="H5" s="184"/>
+      <c r="I5" s="194" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="102"/>
-      <c r="K5" s="57"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="65"/>
-      <c r="N5" s="65"/>
-      <c r="O5" s="65"/>
-      <c r="P5" s="65"/>
-      <c r="Q5" s="66"/>
-      <c r="R5" s="108" t="s">
+      <c r="J5" s="162"/>
+      <c r="K5" s="165"/>
+      <c r="L5" s="166"/>
+      <c r="M5" s="166"/>
+      <c r="N5" s="166"/>
+      <c r="O5" s="166"/>
+      <c r="P5" s="166"/>
+      <c r="Q5" s="167"/>
+      <c r="R5" s="174" t="s">
         <v>11</v>
       </c>
       <c r="S5" s="2"/>
-      <c r="T5" s="111"/>
+      <c r="T5" s="177"/>
     </row>
     <row r="6" spans="1:25" ht="25.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="64"/>
-      <c r="B6" s="67"/>
-      <c r="C6" s="68"/>
-      <c r="D6" s="68"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="69"/>
-      <c r="G6" s="60"/>
-      <c r="H6" s="114"/>
-      <c r="I6" s="100"/>
-      <c r="J6" s="103"/>
-      <c r="K6" s="105"/>
-      <c r="L6" s="106"/>
-      <c r="M6" s="106"/>
-      <c r="N6" s="106"/>
-      <c r="O6" s="106"/>
-      <c r="P6" s="106"/>
-      <c r="Q6" s="107"/>
-      <c r="R6" s="109"/>
+      <c r="A6" s="203"/>
+      <c r="B6" s="204"/>
+      <c r="C6" s="205"/>
+      <c r="D6" s="205"/>
+      <c r="E6" s="205"/>
+      <c r="F6" s="206"/>
+      <c r="G6" s="191"/>
+      <c r="H6" s="192"/>
+      <c r="I6" s="195"/>
+      <c r="J6" s="163"/>
+      <c r="K6" s="168"/>
+      <c r="L6" s="169"/>
+      <c r="M6" s="169"/>
+      <c r="N6" s="169"/>
+      <c r="O6" s="169"/>
+      <c r="P6" s="169"/>
+      <c r="Q6" s="170"/>
+      <c r="R6" s="175"/>
       <c r="S6" s="3"/>
-      <c r="T6" s="112"/>
+      <c r="T6" s="178"/>
     </row>
     <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="63" t="s">
+      <c r="A7" s="196" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="139"/>
-      <c r="C7" s="84"/>
-      <c r="D7" s="84"/>
-      <c r="E7" s="84"/>
-      <c r="F7" s="140"/>
-      <c r="G7" s="97" t="s">
+      <c r="B7" s="188"/>
+      <c r="C7" s="189"/>
+      <c r="D7" s="189"/>
+      <c r="E7" s="189"/>
+      <c r="F7" s="190"/>
+      <c r="G7" s="193" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="98"/>
-      <c r="I7" s="101"/>
-      <c r="J7" s="104"/>
-      <c r="K7" s="67"/>
-      <c r="L7" s="68"/>
-      <c r="M7" s="68"/>
-      <c r="N7" s="68"/>
-      <c r="O7" s="68"/>
-      <c r="P7" s="68"/>
-      <c r="Q7" s="69"/>
-      <c r="R7" s="110"/>
+      <c r="H7" s="184"/>
+      <c r="I7" s="232"/>
+      <c r="J7" s="233"/>
+      <c r="K7" s="204"/>
+      <c r="L7" s="205"/>
+      <c r="M7" s="205"/>
+      <c r="N7" s="205"/>
+      <c r="O7" s="205"/>
+      <c r="P7" s="205"/>
+      <c r="Q7" s="206"/>
+      <c r="R7" s="234"/>
       <c r="S7" s="4"/>
-      <c r="T7" s="113"/>
+      <c r="T7" s="235"/>
       <c r="Y7" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:25" ht="25.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="141"/>
-      <c r="B8" s="60"/>
-      <c r="C8" s="85"/>
-      <c r="D8" s="85"/>
-      <c r="E8" s="85"/>
-      <c r="F8" s="114"/>
-      <c r="G8" s="60"/>
-      <c r="H8" s="114"/>
-      <c r="I8" s="99" t="s">
+      <c r="A8" s="197"/>
+      <c r="B8" s="191"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="60"/>
+      <c r="E8" s="60"/>
+      <c r="F8" s="192"/>
+      <c r="G8" s="191"/>
+      <c r="H8" s="192"/>
+      <c r="I8" s="194" t="s">
         <v>15</v>
       </c>
-      <c r="J8" s="102"/>
-      <c r="K8" s="57"/>
-      <c r="L8" s="65"/>
-      <c r="M8" s="65"/>
-      <c r="N8" s="65"/>
-      <c r="O8" s="65"/>
-      <c r="P8" s="65"/>
-      <c r="Q8" s="66"/>
-      <c r="R8" s="108" t="s">
+      <c r="J8" s="162"/>
+      <c r="K8" s="165"/>
+      <c r="L8" s="166"/>
+      <c r="M8" s="166"/>
+      <c r="N8" s="166"/>
+      <c r="O8" s="166"/>
+      <c r="P8" s="166"/>
+      <c r="Q8" s="167"/>
+      <c r="R8" s="174" t="s">
         <v>16</v>
       </c>
       <c r="S8" s="2"/>
-      <c r="T8" s="111"/>
+      <c r="T8" s="177"/>
       <c r="Y8" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="25.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="132" t="s">
+      <c r="A9" s="180" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="133"/>
-      <c r="C9" s="133"/>
-      <c r="D9" s="134">
+      <c r="B9" s="181"/>
+      <c r="C9" s="181"/>
+      <c r="D9" s="182">
         <v>1</v>
       </c>
-      <c r="E9" s="134"/>
-      <c r="F9" s="134"/>
-      <c r="G9" s="135" t="s">
+      <c r="E9" s="182"/>
+      <c r="F9" s="182"/>
+      <c r="G9" s="183" t="s">
         <v>19</v>
       </c>
-      <c r="H9" s="98"/>
-      <c r="I9" s="100"/>
-      <c r="J9" s="103"/>
-      <c r="K9" s="105"/>
-      <c r="L9" s="106"/>
-      <c r="M9" s="106"/>
-      <c r="N9" s="106"/>
-      <c r="O9" s="106"/>
-      <c r="P9" s="106"/>
-      <c r="Q9" s="107"/>
-      <c r="R9" s="109"/>
+      <c r="H9" s="184"/>
+      <c r="I9" s="195"/>
+      <c r="J9" s="163"/>
+      <c r="K9" s="168"/>
+      <c r="L9" s="169"/>
+      <c r="M9" s="169"/>
+      <c r="N9" s="169"/>
+      <c r="O9" s="169"/>
+      <c r="P9" s="169"/>
+      <c r="Q9" s="170"/>
+      <c r="R9" s="175"/>
       <c r="S9" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="T9" s="112"/>
+      <c r="T9" s="178"/>
       <c r="Y9" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="25.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="136" t="s">
+      <c r="A10" s="185" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="133"/>
-      <c r="C10" s="133"/>
-      <c r="D10" s="134">
+      <c r="B10" s="181"/>
+      <c r="C10" s="181"/>
+      <c r="D10" s="182">
         <v>1</v>
       </c>
-      <c r="E10" s="134"/>
-      <c r="F10" s="134"/>
-      <c r="G10" s="137">
+      <c r="E10" s="182"/>
+      <c r="F10" s="182"/>
+      <c r="G10" s="186">
         <v>2</v>
       </c>
-      <c r="H10" s="138"/>
-      <c r="I10" s="100"/>
-      <c r="J10" s="126"/>
-      <c r="K10" s="127"/>
-      <c r="L10" s="128"/>
-      <c r="M10" s="128"/>
-      <c r="N10" s="128"/>
-      <c r="O10" s="128"/>
-      <c r="P10" s="128"/>
-      <c r="Q10" s="129"/>
-      <c r="R10" s="130"/>
+      <c r="H10" s="187"/>
+      <c r="I10" s="195"/>
+      <c r="J10" s="164"/>
+      <c r="K10" s="171"/>
+      <c r="L10" s="172"/>
+      <c r="M10" s="172"/>
+      <c r="N10" s="172"/>
+      <c r="O10" s="172"/>
+      <c r="P10" s="172"/>
+      <c r="Q10" s="173"/>
+      <c r="R10" s="176"/>
       <c r="S10" s="6"/>
-      <c r="T10" s="131"/>
+      <c r="T10" s="179"/>
       <c r="Y10" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="115"/>
-      <c r="B11" s="115"/>
-      <c r="C11" s="116" t="s">
+      <c r="A11" s="154"/>
+      <c r="B11" s="154"/>
+      <c r="C11" s="155" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="117"/>
-      <c r="E11" s="118"/>
-      <c r="F11" s="116" t="s">
+      <c r="D11" s="156"/>
+      <c r="E11" s="157"/>
+      <c r="F11" s="155" t="s">
         <v>24</v>
       </c>
-      <c r="G11" s="117"/>
-      <c r="H11" s="117"/>
-      <c r="I11" s="118"/>
-      <c r="J11" s="117"/>
-      <c r="K11" s="122" t="s">
+      <c r="G11" s="156"/>
+      <c r="H11" s="156"/>
+      <c r="I11" s="157"/>
+      <c r="J11" s="156"/>
+      <c r="K11" s="158" t="s">
         <v>25</v>
       </c>
-      <c r="L11" s="123"/>
-      <c r="M11" s="116" t="s">
+      <c r="L11" s="159"/>
+      <c r="M11" s="155" t="s">
         <v>26</v>
       </c>
-      <c r="N11" s="117"/>
-      <c r="O11" s="117"/>
-      <c r="P11" s="117"/>
-      <c r="Q11" s="117"/>
-      <c r="R11" s="117"/>
-      <c r="S11" s="117"/>
-      <c r="T11" s="118"/>
+      <c r="N11" s="156"/>
+      <c r="O11" s="156"/>
+      <c r="P11" s="156"/>
+      <c r="Q11" s="156"/>
+      <c r="R11" s="156"/>
+      <c r="S11" s="156"/>
+      <c r="T11" s="157"/>
       <c r="V11" s="7"/>
       <c r="Y11" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A12" s="115"/>
-      <c r="B12" s="115"/>
-      <c r="C12" s="119"/>
-      <c r="D12" s="120"/>
-      <c r="E12" s="121"/>
-      <c r="F12" s="119"/>
-      <c r="G12" s="120"/>
-      <c r="H12" s="120"/>
-      <c r="I12" s="121"/>
-      <c r="J12" s="120"/>
-      <c r="K12" s="124"/>
-      <c r="L12" s="125"/>
-      <c r="M12" s="119"/>
-      <c r="N12" s="120"/>
-      <c r="O12" s="120"/>
-      <c r="P12" s="120"/>
-      <c r="Q12" s="120"/>
-      <c r="R12" s="120"/>
-      <c r="S12" s="120"/>
-      <c r="T12" s="121"/>
+      <c r="A12" s="154"/>
+      <c r="B12" s="154"/>
+      <c r="C12" s="83"/>
+      <c r="D12" s="84"/>
+      <c r="E12" s="126"/>
+      <c r="F12" s="83"/>
+      <c r="G12" s="84"/>
+      <c r="H12" s="84"/>
+      <c r="I12" s="126"/>
+      <c r="J12" s="84"/>
+      <c r="K12" s="160"/>
+      <c r="L12" s="161"/>
+      <c r="M12" s="83"/>
+      <c r="N12" s="84"/>
+      <c r="O12" s="84"/>
+      <c r="P12" s="84"/>
+      <c r="Q12" s="84"/>
+      <c r="R12" s="84"/>
+      <c r="S12" s="84"/>
+      <c r="T12" s="126"/>
       <c r="Y12" s="6" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="156" t="s">
+      <c r="A13" s="54" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="157"/>
-      <c r="C13" s="158" t="s">
+      <c r="B13" s="125"/>
+      <c r="C13" s="145" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="142" t="s">
+      <c r="D13" s="109" t="s">
         <v>31</v>
       </c>
-      <c r="E13" s="143"/>
-      <c r="F13" s="160" t="s">
+      <c r="E13" s="111"/>
+      <c r="F13" s="147" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="161"/>
-      <c r="H13" s="161"/>
-      <c r="I13" s="162"/>
-      <c r="J13" s="166"/>
-      <c r="K13" s="158" t="s">
+      <c r="G13" s="148"/>
+      <c r="H13" s="148"/>
+      <c r="I13" s="149"/>
+      <c r="J13" s="110"/>
+      <c r="K13" s="145" t="s">
         <v>33</v>
       </c>
-      <c r="L13" s="55" t="s">
+      <c r="L13" s="134" t="s">
         <v>34</v>
       </c>
-      <c r="M13" s="142" t="s">
+      <c r="M13" s="109" t="s">
         <v>35</v>
       </c>
-      <c r="N13" s="143"/>
-      <c r="O13" s="142" t="s">
+      <c r="N13" s="111"/>
+      <c r="O13" s="109" t="s">
         <v>36</v>
       </c>
-      <c r="P13" s="143"/>
-      <c r="Q13" s="142" t="s">
+      <c r="P13" s="111"/>
+      <c r="Q13" s="109" t="s">
         <v>37</v>
       </c>
-      <c r="R13" s="143"/>
-      <c r="S13" s="142" t="s">
+      <c r="R13" s="111"/>
+      <c r="S13" s="109" t="s">
         <v>38</v>
       </c>
-      <c r="T13" s="143"/>
+      <c r="T13" s="111"/>
     </row>
     <row r="14" spans="1:25" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="144"/>
-      <c r="B14" s="145"/>
-      <c r="C14" s="159"/>
-      <c r="D14" s="144"/>
-      <c r="E14" s="145"/>
-      <c r="F14" s="163"/>
-      <c r="G14" s="164"/>
-      <c r="H14" s="164"/>
-      <c r="I14" s="165"/>
-      <c r="J14" s="167"/>
-      <c r="K14" s="159"/>
-      <c r="L14" s="168"/>
-      <c r="M14" s="144"/>
-      <c r="N14" s="145"/>
-      <c r="O14" s="144"/>
-      <c r="P14" s="145"/>
-      <c r="Q14" s="144"/>
-      <c r="R14" s="145"/>
-      <c r="S14" s="144"/>
-      <c r="T14" s="145"/>
+      <c r="A14" s="136"/>
+      <c r="B14" s="137"/>
+      <c r="C14" s="146"/>
+      <c r="D14" s="136"/>
+      <c r="E14" s="137"/>
+      <c r="F14" s="150"/>
+      <c r="G14" s="151"/>
+      <c r="H14" s="151"/>
+      <c r="I14" s="152"/>
+      <c r="J14" s="153"/>
+      <c r="K14" s="146"/>
+      <c r="L14" s="135"/>
+      <c r="M14" s="136"/>
+      <c r="N14" s="137"/>
+      <c r="O14" s="136"/>
+      <c r="P14" s="137"/>
+      <c r="Q14" s="136"/>
+      <c r="R14" s="137"/>
+      <c r="S14" s="136"/>
+      <c r="T14" s="137"/>
       <c r="Y14" s="6" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:25" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="146"/>
-      <c r="B15" s="147"/>
+      <c r="A15" s="138"/>
+      <c r="B15" s="139"/>
       <c r="C15" s="8"/>
-      <c r="D15" s="148"/>
-      <c r="E15" s="149"/>
-      <c r="F15" s="150"/>
-      <c r="G15" s="151"/>
-      <c r="H15" s="151"/>
-      <c r="I15" s="152"/>
-      <c r="J15" s="153"/>
+      <c r="D15" s="140"/>
+      <c r="E15" s="141"/>
+      <c r="F15" s="236"/>
+      <c r="G15" s="237"/>
+      <c r="H15" s="237"/>
+      <c r="I15" s="238"/>
+      <c r="J15" s="142"/>
       <c r="K15" s="9"/>
       <c r="L15" s="10"/>
       <c r="M15" s="11"/>
@@ -4211,16 +4215,16 @@
       </c>
     </row>
     <row r="16" spans="1:25" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="51"/>
-      <c r="B16" s="52"/>
+      <c r="A16" s="130"/>
+      <c r="B16" s="131"/>
       <c r="C16" s="13"/>
-      <c r="D16" s="53"/>
-      <c r="E16" s="54"/>
-      <c r="F16" s="48"/>
-      <c r="G16" s="49"/>
-      <c r="H16" s="49"/>
-      <c r="I16" s="50"/>
-      <c r="J16" s="154"/>
+      <c r="D16" s="132"/>
+      <c r="E16" s="133"/>
+      <c r="F16" s="106"/>
+      <c r="G16" s="107"/>
+      <c r="H16" s="107"/>
+      <c r="I16" s="108"/>
+      <c r="J16" s="143"/>
       <c r="K16" s="14"/>
       <c r="L16" s="15"/>
       <c r="M16" s="16"/>
@@ -4236,16 +4240,16 @@
       </c>
     </row>
     <row r="17" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51"/>
-      <c r="B17" s="52"/>
+      <c r="A17" s="130"/>
+      <c r="B17" s="131"/>
       <c r="C17" s="13"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="54"/>
-      <c r="F17" s="48"/>
-      <c r="G17" s="49"/>
-      <c r="H17" s="49"/>
-      <c r="I17" s="50"/>
-      <c r="J17" s="154"/>
+      <c r="D17" s="132"/>
+      <c r="E17" s="133"/>
+      <c r="F17" s="106"/>
+      <c r="G17" s="107"/>
+      <c r="H17" s="107"/>
+      <c r="I17" s="108"/>
+      <c r="J17" s="143"/>
       <c r="K17" s="14"/>
       <c r="L17" s="15"/>
       <c r="M17" s="16"/>
@@ -4258,16 +4262,16 @@
       <c r="T17" s="45"/>
     </row>
     <row r="18" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="51"/>
-      <c r="B18" s="52"/>
+      <c r="A18" s="130"/>
+      <c r="B18" s="131"/>
       <c r="C18" s="13"/>
-      <c r="D18" s="53"/>
-      <c r="E18" s="54"/>
-      <c r="F18" s="48"/>
-      <c r="G18" s="49"/>
-      <c r="H18" s="49"/>
-      <c r="I18" s="50"/>
-      <c r="J18" s="154"/>
+      <c r="D18" s="132"/>
+      <c r="E18" s="133"/>
+      <c r="F18" s="106"/>
+      <c r="G18" s="107"/>
+      <c r="H18" s="107"/>
+      <c r="I18" s="108"/>
+      <c r="J18" s="143"/>
       <c r="K18" s="14"/>
       <c r="L18" s="15"/>
       <c r="M18" s="16"/>
@@ -4280,16 +4284,16 @@
       <c r="T18" s="45"/>
     </row>
     <row r="19" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="51"/>
-      <c r="B19" s="52"/>
+      <c r="A19" s="130"/>
+      <c r="B19" s="131"/>
       <c r="C19" s="13"/>
-      <c r="D19" s="53"/>
-      <c r="E19" s="54"/>
-      <c r="F19" s="48"/>
-      <c r="G19" s="49"/>
-      <c r="H19" s="49"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="154"/>
+      <c r="D19" s="132"/>
+      <c r="E19" s="133"/>
+      <c r="F19" s="106"/>
+      <c r="G19" s="107"/>
+      <c r="H19" s="107"/>
+      <c r="I19" s="108"/>
+      <c r="J19" s="143"/>
       <c r="K19" s="14"/>
       <c r="L19" s="15"/>
       <c r="M19" s="16"/>
@@ -4302,16 +4306,16 @@
       <c r="T19" s="45"/>
     </row>
     <row r="20" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="51"/>
-      <c r="B20" s="52"/>
+      <c r="A20" s="130"/>
+      <c r="B20" s="131"/>
       <c r="C20" s="13"/>
-      <c r="D20" s="53"/>
-      <c r="E20" s="54"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="49"/>
-      <c r="H20" s="49"/>
-      <c r="I20" s="50"/>
-      <c r="J20" s="154"/>
+      <c r="D20" s="132"/>
+      <c r="E20" s="133"/>
+      <c r="F20" s="106"/>
+      <c r="G20" s="107"/>
+      <c r="H20" s="107"/>
+      <c r="I20" s="108"/>
+      <c r="J20" s="143"/>
       <c r="K20" s="14"/>
       <c r="L20" s="15"/>
       <c r="M20" s="16"/>
@@ -4324,16 +4328,16 @@
       <c r="T20" s="45"/>
     </row>
     <row r="21" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="51"/>
-      <c r="B21" s="52"/>
+      <c r="A21" s="130"/>
+      <c r="B21" s="131"/>
       <c r="C21" s="13"/>
-      <c r="D21" s="53"/>
-      <c r="E21" s="54"/>
-      <c r="F21" s="48"/>
-      <c r="G21" s="49"/>
-      <c r="H21" s="49"/>
-      <c r="I21" s="50"/>
-      <c r="J21" s="154"/>
+      <c r="D21" s="132"/>
+      <c r="E21" s="133"/>
+      <c r="F21" s="106"/>
+      <c r="G21" s="107"/>
+      <c r="H21" s="107"/>
+      <c r="I21" s="108"/>
+      <c r="J21" s="143"/>
       <c r="K21" s="14"/>
       <c r="L21" s="15"/>
       <c r="M21" s="16"/>
@@ -4346,16 +4350,16 @@
       <c r="T21" s="45"/>
     </row>
     <row r="22" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="51"/>
-      <c r="B22" s="52"/>
+      <c r="A22" s="130"/>
+      <c r="B22" s="131"/>
       <c r="C22" s="13"/>
-      <c r="D22" s="53"/>
-      <c r="E22" s="54"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="49"/>
-      <c r="H22" s="49"/>
-      <c r="I22" s="50"/>
-      <c r="J22" s="154"/>
+      <c r="D22" s="132"/>
+      <c r="E22" s="133"/>
+      <c r="F22" s="106"/>
+      <c r="G22" s="107"/>
+      <c r="H22" s="107"/>
+      <c r="I22" s="108"/>
+      <c r="J22" s="143"/>
       <c r="K22" s="14"/>
       <c r="L22" s="15"/>
       <c r="M22" s="16"/>
@@ -4368,16 +4372,16 @@
       <c r="T22" s="45"/>
     </row>
     <row r="23" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="51"/>
-      <c r="B23" s="52"/>
+      <c r="A23" s="130"/>
+      <c r="B23" s="131"/>
       <c r="C23" s="13"/>
-      <c r="D23" s="53"/>
-      <c r="E23" s="54"/>
-      <c r="F23" s="48"/>
-      <c r="G23" s="49"/>
-      <c r="H23" s="49"/>
-      <c r="I23" s="50"/>
-      <c r="J23" s="154"/>
+      <c r="D23" s="132"/>
+      <c r="E23" s="133"/>
+      <c r="F23" s="106"/>
+      <c r="G23" s="107"/>
+      <c r="H23" s="107"/>
+      <c r="I23" s="108"/>
+      <c r="J23" s="143"/>
       <c r="K23" s="14"/>
       <c r="L23" s="15"/>
       <c r="M23" s="16"/>
@@ -4390,16 +4394,16 @@
       <c r="T23" s="45"/>
     </row>
     <row r="24" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="51"/>
-      <c r="B24" s="52"/>
+      <c r="A24" s="130"/>
+      <c r="B24" s="131"/>
       <c r="C24" s="13"/>
-      <c r="D24" s="53"/>
-      <c r="E24" s="54"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="49"/>
-      <c r="H24" s="49"/>
-      <c r="I24" s="50"/>
-      <c r="J24" s="154"/>
+      <c r="D24" s="132"/>
+      <c r="E24" s="133"/>
+      <c r="F24" s="106"/>
+      <c r="G24" s="107"/>
+      <c r="H24" s="107"/>
+      <c r="I24" s="108"/>
+      <c r="J24" s="143"/>
       <c r="K24" s="14"/>
       <c r="L24" s="15"/>
       <c r="M24" s="16"/>
@@ -4412,16 +4416,16 @@
       <c r="T24" s="45"/>
     </row>
     <row r="25" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="51"/>
-      <c r="B25" s="52"/>
+      <c r="A25" s="130"/>
+      <c r="B25" s="131"/>
       <c r="C25" s="13"/>
-      <c r="D25" s="53"/>
-      <c r="E25" s="54"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="49"/>
-      <c r="H25" s="49"/>
-      <c r="I25" s="50"/>
-      <c r="J25" s="154"/>
+      <c r="D25" s="132"/>
+      <c r="E25" s="133"/>
+      <c r="F25" s="106"/>
+      <c r="G25" s="107"/>
+      <c r="H25" s="107"/>
+      <c r="I25" s="108"/>
+      <c r="J25" s="143"/>
       <c r="K25" s="14"/>
       <c r="L25" s="15"/>
       <c r="M25" s="16"/>
@@ -4434,16 +4438,16 @@
       <c r="T25" s="45"/>
     </row>
     <row r="26" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="51"/>
-      <c r="B26" s="52"/>
+      <c r="A26" s="130"/>
+      <c r="B26" s="131"/>
       <c r="C26" s="13"/>
-      <c r="D26" s="53"/>
-      <c r="E26" s="54"/>
-      <c r="F26" s="48"/>
-      <c r="G26" s="49"/>
-      <c r="H26" s="49"/>
-      <c r="I26" s="50"/>
-      <c r="J26" s="154"/>
+      <c r="D26" s="132"/>
+      <c r="E26" s="133"/>
+      <c r="F26" s="106"/>
+      <c r="G26" s="107"/>
+      <c r="H26" s="107"/>
+      <c r="I26" s="108"/>
+      <c r="J26" s="143"/>
       <c r="K26" s="14"/>
       <c r="L26" s="15"/>
       <c r="M26" s="16"/>
@@ -4456,16 +4460,16 @@
       <c r="T26" s="45"/>
     </row>
     <row r="27" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="51"/>
-      <c r="B27" s="52"/>
+      <c r="A27" s="130"/>
+      <c r="B27" s="131"/>
       <c r="C27" s="13"/>
-      <c r="D27" s="53"/>
-      <c r="E27" s="54"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="49"/>
-      <c r="H27" s="49"/>
-      <c r="I27" s="50"/>
-      <c r="J27" s="154"/>
+      <c r="D27" s="132"/>
+      <c r="E27" s="133"/>
+      <c r="F27" s="106"/>
+      <c r="G27" s="107"/>
+      <c r="H27" s="107"/>
+      <c r="I27" s="108"/>
+      <c r="J27" s="143"/>
       <c r="K27" s="14"/>
       <c r="L27" s="15"/>
       <c r="M27" s="16"/>
@@ -4478,16 +4482,16 @@
       <c r="T27" s="45"/>
     </row>
     <row r="28" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="51"/>
-      <c r="B28" s="52"/>
+      <c r="A28" s="130"/>
+      <c r="B28" s="131"/>
       <c r="C28" s="13"/>
-      <c r="D28" s="53"/>
-      <c r="E28" s="54"/>
-      <c r="F28" s="48"/>
-      <c r="G28" s="49"/>
-      <c r="H28" s="49"/>
-      <c r="I28" s="50"/>
-      <c r="J28" s="154"/>
+      <c r="D28" s="132"/>
+      <c r="E28" s="133"/>
+      <c r="F28" s="106"/>
+      <c r="G28" s="107"/>
+      <c r="H28" s="107"/>
+      <c r="I28" s="108"/>
+      <c r="J28" s="143"/>
       <c r="K28" s="14"/>
       <c r="L28" s="15"/>
       <c r="M28" s="37"/>
@@ -4500,16 +4504,16 @@
       <c r="T28" s="45"/>
     </row>
     <row r="29" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="51"/>
-      <c r="B29" s="52"/>
+      <c r="A29" s="130"/>
+      <c r="B29" s="131"/>
       <c r="C29" s="13"/>
-      <c r="D29" s="53"/>
-      <c r="E29" s="54"/>
-      <c r="F29" s="48"/>
-      <c r="G29" s="49"/>
-      <c r="H29" s="49"/>
-      <c r="I29" s="50"/>
-      <c r="J29" s="154"/>
+      <c r="D29" s="132"/>
+      <c r="E29" s="133"/>
+      <c r="F29" s="106"/>
+      <c r="G29" s="107"/>
+      <c r="H29" s="107"/>
+      <c r="I29" s="108"/>
+      <c r="J29" s="143"/>
       <c r="K29" s="14"/>
       <c r="L29" s="15"/>
       <c r="M29" s="37"/>
@@ -4522,16 +4526,16 @@
       <c r="T29" s="45"/>
     </row>
     <row r="30" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="51"/>
-      <c r="B30" s="52"/>
+      <c r="A30" s="130"/>
+      <c r="B30" s="131"/>
       <c r="C30" s="13"/>
-      <c r="D30" s="53"/>
-      <c r="E30" s="54"/>
-      <c r="F30" s="48"/>
-      <c r="G30" s="49"/>
-      <c r="H30" s="49"/>
-      <c r="I30" s="50"/>
-      <c r="J30" s="154"/>
+      <c r="D30" s="132"/>
+      <c r="E30" s="133"/>
+      <c r="F30" s="106"/>
+      <c r="G30" s="107"/>
+      <c r="H30" s="107"/>
+      <c r="I30" s="108"/>
+      <c r="J30" s="143"/>
       <c r="K30" s="14"/>
       <c r="L30" s="15"/>
       <c r="M30" s="37"/>
@@ -4544,16 +4548,16 @@
       <c r="T30" s="45"/>
     </row>
     <row r="31" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="51"/>
-      <c r="B31" s="52"/>
+      <c r="A31" s="130"/>
+      <c r="B31" s="131"/>
       <c r="C31" s="13"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="54"/>
-      <c r="F31" s="48"/>
-      <c r="G31" s="49"/>
-      <c r="H31" s="49"/>
-      <c r="I31" s="50"/>
-      <c r="J31" s="154"/>
+      <c r="D31" s="132"/>
+      <c r="E31" s="133"/>
+      <c r="F31" s="106"/>
+      <c r="G31" s="107"/>
+      <c r="H31" s="107"/>
+      <c r="I31" s="108"/>
+      <c r="J31" s="143"/>
       <c r="K31" s="14"/>
       <c r="L31" s="15"/>
       <c r="M31" s="37"/>
@@ -4566,16 +4570,16 @@
       <c r="T31" s="45"/>
     </row>
     <row r="32" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="51"/>
-      <c r="B32" s="52"/>
+      <c r="A32" s="130"/>
+      <c r="B32" s="131"/>
       <c r="C32" s="13"/>
-      <c r="D32" s="53"/>
-      <c r="E32" s="54"/>
-      <c r="F32" s="48"/>
-      <c r="G32" s="49"/>
-      <c r="H32" s="49"/>
-      <c r="I32" s="50"/>
-      <c r="J32" s="154"/>
+      <c r="D32" s="132"/>
+      <c r="E32" s="133"/>
+      <c r="F32" s="106"/>
+      <c r="G32" s="107"/>
+      <c r="H32" s="107"/>
+      <c r="I32" s="108"/>
+      <c r="J32" s="143"/>
       <c r="K32" s="14"/>
       <c r="L32" s="15"/>
       <c r="M32" s="37"/>
@@ -4588,16 +4592,16 @@
       <c r="T32" s="45"/>
     </row>
     <row r="33" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="51"/>
-      <c r="B33" s="52"/>
+      <c r="A33" s="130"/>
+      <c r="B33" s="131"/>
       <c r="C33" s="13"/>
-      <c r="D33" s="53"/>
-      <c r="E33" s="54"/>
-      <c r="F33" s="48"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="50"/>
-      <c r="J33" s="154"/>
+      <c r="D33" s="132"/>
+      <c r="E33" s="133"/>
+      <c r="F33" s="106"/>
+      <c r="G33" s="107"/>
+      <c r="H33" s="107"/>
+      <c r="I33" s="108"/>
+      <c r="J33" s="143"/>
       <c r="K33" s="14"/>
       <c r="L33" s="15"/>
       <c r="M33" s="37"/>
@@ -4610,16 +4614,16 @@
       <c r="T33" s="45"/>
     </row>
     <row r="34" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="51"/>
-      <c r="B34" s="52"/>
+      <c r="A34" s="130"/>
+      <c r="B34" s="131"/>
       <c r="C34" s="13"/>
-      <c r="D34" s="53"/>
-      <c r="E34" s="54"/>
-      <c r="F34" s="48"/>
-      <c r="G34" s="49"/>
-      <c r="H34" s="49"/>
-      <c r="I34" s="50"/>
-      <c r="J34" s="154"/>
+      <c r="D34" s="132"/>
+      <c r="E34" s="133"/>
+      <c r="F34" s="106"/>
+      <c r="G34" s="107"/>
+      <c r="H34" s="107"/>
+      <c r="I34" s="108"/>
+      <c r="J34" s="143"/>
       <c r="K34" s="14"/>
       <c r="L34" s="15"/>
       <c r="M34" s="37"/>
@@ -4632,16 +4636,16 @@
       <c r="T34" s="45"/>
     </row>
     <row r="35" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="51"/>
-      <c r="B35" s="52"/>
+      <c r="A35" s="130"/>
+      <c r="B35" s="131"/>
       <c r="C35" s="13"/>
-      <c r="D35" s="53"/>
-      <c r="E35" s="54"/>
-      <c r="F35" s="48"/>
-      <c r="G35" s="49"/>
-      <c r="H35" s="49"/>
-      <c r="I35" s="50"/>
-      <c r="J35" s="154"/>
+      <c r="D35" s="132"/>
+      <c r="E35" s="133"/>
+      <c r="F35" s="106"/>
+      <c r="G35" s="107"/>
+      <c r="H35" s="107"/>
+      <c r="I35" s="108"/>
+      <c r="J35" s="143"/>
       <c r="K35" s="14"/>
       <c r="L35" s="15"/>
       <c r="M35" s="37"/>
@@ -4654,16 +4658,16 @@
       <c r="T35" s="45"/>
     </row>
     <row r="36" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="51"/>
-      <c r="B36" s="52"/>
+      <c r="A36" s="130"/>
+      <c r="B36" s="131"/>
       <c r="C36" s="13"/>
-      <c r="D36" s="53"/>
-      <c r="E36" s="54"/>
-      <c r="F36" s="48"/>
-      <c r="G36" s="49"/>
-      <c r="H36" s="49"/>
-      <c r="I36" s="50"/>
-      <c r="J36" s="154"/>
+      <c r="D36" s="132"/>
+      <c r="E36" s="133"/>
+      <c r="F36" s="106"/>
+      <c r="G36" s="107"/>
+      <c r="H36" s="107"/>
+      <c r="I36" s="108"/>
+      <c r="J36" s="143"/>
       <c r="K36" s="14"/>
       <c r="L36" s="15"/>
       <c r="M36" s="37"/>
@@ -4676,16 +4680,16 @@
       <c r="T36" s="45"/>
     </row>
     <row r="37" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="51"/>
-      <c r="B37" s="52"/>
+      <c r="A37" s="130"/>
+      <c r="B37" s="131"/>
       <c r="C37" s="13"/>
-      <c r="D37" s="53"/>
-      <c r="E37" s="54"/>
-      <c r="F37" s="48"/>
-      <c r="G37" s="49"/>
-      <c r="H37" s="49"/>
-      <c r="I37" s="50"/>
-      <c r="J37" s="154"/>
+      <c r="D37" s="132"/>
+      <c r="E37" s="133"/>
+      <c r="F37" s="106"/>
+      <c r="G37" s="107"/>
+      <c r="H37" s="107"/>
+      <c r="I37" s="108"/>
+      <c r="J37" s="143"/>
       <c r="K37" s="14"/>
       <c r="L37" s="15"/>
       <c r="M37" s="37"/>
@@ -4698,16 +4702,16 @@
       <c r="T37" s="45"/>
     </row>
     <row r="38" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="51"/>
-      <c r="B38" s="52"/>
+      <c r="A38" s="130"/>
+      <c r="B38" s="131"/>
       <c r="C38" s="13"/>
-      <c r="D38" s="53"/>
-      <c r="E38" s="54"/>
-      <c r="F38" s="48"/>
-      <c r="G38" s="49"/>
-      <c r="H38" s="49"/>
-      <c r="I38" s="50"/>
-      <c r="J38" s="154"/>
+      <c r="D38" s="132"/>
+      <c r="E38" s="133"/>
+      <c r="F38" s="106"/>
+      <c r="G38" s="107"/>
+      <c r="H38" s="107"/>
+      <c r="I38" s="108"/>
+      <c r="J38" s="143"/>
       <c r="K38" s="14"/>
       <c r="L38" s="15"/>
       <c r="M38" s="37"/>
@@ -4720,16 +4724,16 @@
       <c r="T38" s="45"/>
     </row>
     <row r="39" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="51"/>
-      <c r="B39" s="52"/>
+      <c r="A39" s="130"/>
+      <c r="B39" s="131"/>
       <c r="C39" s="13"/>
-      <c r="D39" s="53"/>
-      <c r="E39" s="54"/>
-      <c r="F39" s="48"/>
-      <c r="G39" s="49"/>
-      <c r="H39" s="49"/>
-      <c r="I39" s="50"/>
-      <c r="J39" s="154"/>
+      <c r="D39" s="132"/>
+      <c r="E39" s="133"/>
+      <c r="F39" s="106"/>
+      <c r="G39" s="107"/>
+      <c r="H39" s="107"/>
+      <c r="I39" s="108"/>
+      <c r="J39" s="143"/>
       <c r="K39" s="14"/>
       <c r="L39" s="15"/>
       <c r="M39" s="37"/>
@@ -4742,16 +4746,16 @@
       <c r="T39" s="45"/>
     </row>
     <row r="40" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="51"/>
-      <c r="B40" s="52"/>
+      <c r="A40" s="130"/>
+      <c r="B40" s="131"/>
       <c r="C40" s="13"/>
-      <c r="D40" s="53"/>
-      <c r="E40" s="54"/>
-      <c r="F40" s="48"/>
-      <c r="G40" s="49"/>
-      <c r="H40" s="49"/>
-      <c r="I40" s="50"/>
-      <c r="J40" s="154"/>
+      <c r="D40" s="132"/>
+      <c r="E40" s="133"/>
+      <c r="F40" s="106"/>
+      <c r="G40" s="107"/>
+      <c r="H40" s="107"/>
+      <c r="I40" s="108"/>
+      <c r="J40" s="143"/>
       <c r="K40" s="14"/>
       <c r="L40" s="15"/>
       <c r="M40" s="37"/>
@@ -4764,16 +4768,16 @@
       <c r="T40" s="45"/>
     </row>
     <row r="41" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="51"/>
-      <c r="B41" s="52"/>
+      <c r="A41" s="130"/>
+      <c r="B41" s="131"/>
       <c r="C41" s="13"/>
-      <c r="D41" s="53"/>
-      <c r="E41" s="54"/>
-      <c r="F41" s="48"/>
-      <c r="G41" s="49"/>
-      <c r="H41" s="49"/>
-      <c r="I41" s="50"/>
-      <c r="J41" s="154"/>
+      <c r="D41" s="132"/>
+      <c r="E41" s="133"/>
+      <c r="F41" s="106"/>
+      <c r="G41" s="107"/>
+      <c r="H41" s="107"/>
+      <c r="I41" s="108"/>
+      <c r="J41" s="143"/>
       <c r="K41" s="14"/>
       <c r="L41" s="15"/>
       <c r="M41" s="37"/>
@@ -4786,16 +4790,16 @@
       <c r="T41" s="45"/>
     </row>
     <row r="42" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="51"/>
-      <c r="B42" s="52"/>
+      <c r="A42" s="130"/>
+      <c r="B42" s="131"/>
       <c r="C42" s="13"/>
-      <c r="D42" s="53"/>
-      <c r="E42" s="54"/>
-      <c r="F42" s="48"/>
-      <c r="G42" s="49"/>
-      <c r="H42" s="49"/>
-      <c r="I42" s="50"/>
-      <c r="J42" s="154"/>
+      <c r="D42" s="132"/>
+      <c r="E42" s="133"/>
+      <c r="F42" s="106"/>
+      <c r="G42" s="107"/>
+      <c r="H42" s="107"/>
+      <c r="I42" s="108"/>
+      <c r="J42" s="143"/>
       <c r="K42" s="14"/>
       <c r="L42" s="15"/>
       <c r="M42" s="37"/>
@@ -4808,16 +4812,16 @@
       <c r="T42" s="45"/>
     </row>
     <row r="43" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="51"/>
-      <c r="B43" s="52"/>
+      <c r="A43" s="130"/>
+      <c r="B43" s="131"/>
       <c r="C43" s="13"/>
-      <c r="D43" s="53"/>
-      <c r="E43" s="54"/>
-      <c r="F43" s="48"/>
-      <c r="G43" s="49"/>
-      <c r="H43" s="49"/>
-      <c r="I43" s="50"/>
-      <c r="J43" s="154"/>
+      <c r="D43" s="132"/>
+      <c r="E43" s="133"/>
+      <c r="F43" s="106"/>
+      <c r="G43" s="107"/>
+      <c r="H43" s="107"/>
+      <c r="I43" s="108"/>
+      <c r="J43" s="143"/>
       <c r="K43" s="14"/>
       <c r="L43" s="15"/>
       <c r="M43" s="37"/>
@@ -4830,16 +4834,16 @@
       <c r="T43" s="45"/>
     </row>
     <row r="44" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="51"/>
-      <c r="B44" s="52"/>
+      <c r="A44" s="130"/>
+      <c r="B44" s="131"/>
       <c r="C44" s="13"/>
-      <c r="D44" s="53"/>
-      <c r="E44" s="54"/>
-      <c r="F44" s="48"/>
-      <c r="G44" s="49"/>
-      <c r="H44" s="49"/>
-      <c r="I44" s="50"/>
-      <c r="J44" s="154"/>
+      <c r="D44" s="132"/>
+      <c r="E44" s="133"/>
+      <c r="F44" s="106"/>
+      <c r="G44" s="107"/>
+      <c r="H44" s="107"/>
+      <c r="I44" s="108"/>
+      <c r="J44" s="143"/>
       <c r="K44" s="14"/>
       <c r="L44" s="15"/>
       <c r="M44" s="37"/>
@@ -4852,16 +4856,16 @@
       <c r="T44" s="45"/>
     </row>
     <row r="45" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="51"/>
-      <c r="B45" s="52"/>
+      <c r="A45" s="130"/>
+      <c r="B45" s="131"/>
       <c r="C45" s="13"/>
-      <c r="D45" s="53"/>
-      <c r="E45" s="54"/>
-      <c r="F45" s="48"/>
-      <c r="G45" s="49"/>
-      <c r="H45" s="49"/>
-      <c r="I45" s="50"/>
-      <c r="J45" s="154"/>
+      <c r="D45" s="132"/>
+      <c r="E45" s="133"/>
+      <c r="F45" s="106"/>
+      <c r="G45" s="107"/>
+      <c r="H45" s="107"/>
+      <c r="I45" s="108"/>
+      <c r="J45" s="143"/>
       <c r="K45" s="14"/>
       <c r="L45" s="15"/>
       <c r="M45" s="37"/>
@@ -4874,16 +4878,16 @@
       <c r="T45" s="45"/>
     </row>
     <row r="46" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="51"/>
-      <c r="B46" s="52"/>
+      <c r="A46" s="130"/>
+      <c r="B46" s="131"/>
       <c r="C46" s="13"/>
-      <c r="D46" s="53"/>
-      <c r="E46" s="54"/>
-      <c r="F46" s="48"/>
-      <c r="G46" s="49"/>
-      <c r="H46" s="49"/>
-      <c r="I46" s="50"/>
-      <c r="J46" s="154"/>
+      <c r="D46" s="132"/>
+      <c r="E46" s="133"/>
+      <c r="F46" s="106"/>
+      <c r="G46" s="107"/>
+      <c r="H46" s="107"/>
+      <c r="I46" s="108"/>
+      <c r="J46" s="143"/>
       <c r="K46" s="14"/>
       <c r="L46" s="15"/>
       <c r="M46" s="37"/>
@@ -4896,16 +4900,16 @@
       <c r="T46" s="45"/>
     </row>
     <row r="47" spans="1:20" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="51"/>
-      <c r="B47" s="52"/>
+      <c r="A47" s="130"/>
+      <c r="B47" s="131"/>
       <c r="C47" s="13"/>
-      <c r="D47" s="53"/>
-      <c r="E47" s="54"/>
-      <c r="F47" s="48"/>
-      <c r="G47" s="49"/>
-      <c r="H47" s="49"/>
-      <c r="I47" s="50"/>
-      <c r="J47" s="154"/>
+      <c r="D47" s="132"/>
+      <c r="E47" s="133"/>
+      <c r="F47" s="106"/>
+      <c r="G47" s="107"/>
+      <c r="H47" s="107"/>
+      <c r="I47" s="108"/>
+      <c r="J47" s="143"/>
       <c r="K47" s="14"/>
       <c r="L47" s="15"/>
       <c r="M47" s="37"/>
@@ -4918,16 +4922,16 @@
       <c r="T47" s="45"/>
     </row>
     <row r="48" spans="1:20" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="51"/>
-      <c r="B48" s="52"/>
+      <c r="A48" s="130"/>
+      <c r="B48" s="131"/>
       <c r="C48" s="13"/>
-      <c r="D48" s="53"/>
-      <c r="E48" s="54"/>
-      <c r="F48" s="48"/>
-      <c r="G48" s="49"/>
-      <c r="H48" s="49"/>
-      <c r="I48" s="50"/>
-      <c r="J48" s="154"/>
+      <c r="D48" s="132"/>
+      <c r="E48" s="133"/>
+      <c r="F48" s="106"/>
+      <c r="G48" s="107"/>
+      <c r="H48" s="107"/>
+      <c r="I48" s="108"/>
+      <c r="J48" s="143"/>
       <c r="K48" s="14"/>
       <c r="L48" s="15"/>
       <c r="M48" s="37"/>
@@ -4940,16 +4944,16 @@
       <c r="T48" s="45"/>
     </row>
     <row r="49" spans="1:20" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="179"/>
-      <c r="B49" s="180"/>
+      <c r="A49" s="102"/>
+      <c r="B49" s="103"/>
       <c r="C49" s="13"/>
-      <c r="D49" s="181"/>
-      <c r="E49" s="182"/>
-      <c r="F49" s="196"/>
-      <c r="G49" s="197"/>
-      <c r="H49" s="197"/>
-      <c r="I49" s="198"/>
-      <c r="J49" s="155"/>
+      <c r="D49" s="104"/>
+      <c r="E49" s="105"/>
+      <c r="F49" s="127"/>
+      <c r="G49" s="128"/>
+      <c r="H49" s="128"/>
+      <c r="I49" s="129"/>
+      <c r="J49" s="144"/>
       <c r="K49" s="14"/>
       <c r="L49" s="15"/>
       <c r="M49" s="37"/>
@@ -4962,183 +4966,183 @@
       <c r="T49" s="45"/>
     </row>
     <row r="50" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="142" t="s">
+      <c r="A50" s="109" t="s">
         <v>42</v>
       </c>
-      <c r="B50" s="166"/>
-      <c r="C50" s="166"/>
-      <c r="D50" s="166"/>
-      <c r="E50" s="143"/>
-      <c r="F50" s="183" t="s">
+      <c r="B50" s="110"/>
+      <c r="C50" s="110"/>
+      <c r="D50" s="110"/>
+      <c r="E50" s="111"/>
+      <c r="F50" s="112" t="s">
         <v>62</v>
       </c>
-      <c r="G50" s="184"/>
-      <c r="H50" s="184"/>
-      <c r="I50" s="185"/>
-      <c r="J50" s="166"/>
-      <c r="K50" s="173" t="s">
+      <c r="G50" s="113"/>
+      <c r="H50" s="113"/>
+      <c r="I50" s="114"/>
+      <c r="J50" s="110"/>
+      <c r="K50" s="98" t="s">
         <v>38</v>
       </c>
-      <c r="L50" s="175"/>
-      <c r="M50" s="177"/>
-      <c r="N50" s="178"/>
-      <c r="O50" s="177"/>
-      <c r="P50" s="178"/>
-      <c r="Q50" s="177"/>
-      <c r="R50" s="178"/>
-      <c r="S50" s="177"/>
-      <c r="T50" s="204"/>
+      <c r="L50" s="100"/>
+      <c r="M50" s="80"/>
+      <c r="N50" s="94"/>
+      <c r="O50" s="80"/>
+      <c r="P50" s="94"/>
+      <c r="Q50" s="80"/>
+      <c r="R50" s="94"/>
+      <c r="S50" s="80"/>
+      <c r="T50" s="95"/>
     </row>
     <row r="51" spans="1:20" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="156"/>
-      <c r="B51" s="189"/>
-      <c r="C51" s="189"/>
-      <c r="D51" s="189"/>
-      <c r="E51" s="189"/>
-      <c r="F51" s="186"/>
-      <c r="G51" s="187"/>
-      <c r="H51" s="187"/>
-      <c r="I51" s="188"/>
-      <c r="J51" s="189"/>
-      <c r="K51" s="174"/>
-      <c r="L51" s="176"/>
-      <c r="M51" s="177"/>
-      <c r="N51" s="178">
+      <c r="A51" s="54"/>
+      <c r="B51" s="118"/>
+      <c r="C51" s="118"/>
+      <c r="D51" s="118"/>
+      <c r="E51" s="118"/>
+      <c r="F51" s="115"/>
+      <c r="G51" s="116"/>
+      <c r="H51" s="116"/>
+      <c r="I51" s="117"/>
+      <c r="J51" s="118"/>
+      <c r="K51" s="99"/>
+      <c r="L51" s="101"/>
+      <c r="M51" s="80"/>
+      <c r="N51" s="94">
         <f>SUM(N15:N49)</f>
         <v>0</v>
       </c>
-      <c r="O51" s="177"/>
-      <c r="P51" s="178"/>
-      <c r="Q51" s="177"/>
-      <c r="R51" s="178"/>
-      <c r="S51" s="177"/>
-      <c r="T51" s="204"/>
+      <c r="O51" s="80"/>
+      <c r="P51" s="94"/>
+      <c r="Q51" s="80"/>
+      <c r="R51" s="94"/>
+      <c r="S51" s="80"/>
+      <c r="T51" s="95"/>
     </row>
     <row r="52" spans="1:20" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="18" t="s">
         <v>43</v>
       </c>
       <c r="B52" s="3"/>
-      <c r="C52" s="189"/>
-      <c r="D52" s="189"/>
-      <c r="E52" s="189"/>
-      <c r="F52" s="186"/>
-      <c r="G52" s="187"/>
-      <c r="H52" s="187"/>
-      <c r="I52" s="188"/>
-      <c r="J52" s="189"/>
-      <c r="K52" s="169" t="s">
+      <c r="C52" s="118"/>
+      <c r="D52" s="118"/>
+      <c r="E52" s="118"/>
+      <c r="F52" s="115"/>
+      <c r="G52" s="116"/>
+      <c r="H52" s="116"/>
+      <c r="I52" s="117"/>
+      <c r="J52" s="118"/>
+      <c r="K52" s="96" t="s">
         <v>44</v>
       </c>
-      <c r="L52" s="199"/>
-      <c r="M52" s="171"/>
-      <c r="N52" s="171"/>
-      <c r="O52" s="177"/>
-      <c r="P52" s="201"/>
-      <c r="Q52" s="177"/>
-      <c r="R52" s="201"/>
-      <c r="S52" s="177"/>
-      <c r="T52" s="202"/>
+      <c r="L52" s="87"/>
+      <c r="M52" s="88"/>
+      <c r="N52" s="88"/>
+      <c r="O52" s="80"/>
+      <c r="P52" s="91"/>
+      <c r="Q52" s="80"/>
+      <c r="R52" s="91"/>
+      <c r="S52" s="80"/>
+      <c r="T52" s="92"/>
     </row>
     <row r="53" spans="1:20" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="156"/>
-      <c r="B53" s="189"/>
-      <c r="C53" s="189"/>
-      <c r="D53" s="189"/>
-      <c r="E53" s="157"/>
+      <c r="A53" s="54"/>
+      <c r="B53" s="118"/>
+      <c r="C53" s="118"/>
+      <c r="D53" s="118"/>
+      <c r="E53" s="125"/>
       <c r="F53" s="19"/>
       <c r="G53" s="20"/>
-      <c r="H53" s="190"/>
-      <c r="I53" s="191"/>
-      <c r="J53" s="189"/>
-      <c r="K53" s="170"/>
-      <c r="L53" s="200"/>
-      <c r="M53" s="172"/>
-      <c r="N53" s="172"/>
-      <c r="O53" s="177"/>
-      <c r="P53" s="201"/>
-      <c r="Q53" s="177"/>
-      <c r="R53" s="201"/>
-      <c r="S53" s="177"/>
-      <c r="T53" s="203"/>
+      <c r="H53" s="119"/>
+      <c r="I53" s="120"/>
+      <c r="J53" s="118"/>
+      <c r="K53" s="97"/>
+      <c r="L53" s="89"/>
+      <c r="M53" s="90"/>
+      <c r="N53" s="90"/>
+      <c r="O53" s="80"/>
+      <c r="P53" s="91"/>
+      <c r="Q53" s="80"/>
+      <c r="R53" s="91"/>
+      <c r="S53" s="80"/>
+      <c r="T53" s="93"/>
     </row>
     <row r="54" spans="1:20" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="18" t="s">
         <v>45</v>
       </c>
       <c r="B54" s="21"/>
-      <c r="C54" s="189"/>
-      <c r="D54" s="189"/>
-      <c r="E54" s="157"/>
-      <c r="F54" s="156"/>
-      <c r="G54" s="189"/>
-      <c r="H54" s="192" t="s">
+      <c r="C54" s="118"/>
+      <c r="D54" s="118"/>
+      <c r="E54" s="125"/>
+      <c r="F54" s="54"/>
+      <c r="G54" s="118"/>
+      <c r="H54" s="121" t="s">
         <v>46</v>
       </c>
-      <c r="I54" s="193"/>
-      <c r="J54" s="189"/>
+      <c r="I54" s="122"/>
+      <c r="J54" s="118"/>
       <c r="K54" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="L54" s="177"/>
-      <c r="M54" s="177"/>
-      <c r="N54" s="208"/>
-      <c r="O54" s="177"/>
-      <c r="P54" s="205"/>
-      <c r="Q54" s="177"/>
-      <c r="R54" s="205"/>
-      <c r="S54" s="177"/>
-      <c r="T54" s="206"/>
+      <c r="L54" s="80"/>
+      <c r="M54" s="80"/>
+      <c r="N54" s="85"/>
+      <c r="O54" s="80"/>
+      <c r="P54" s="79"/>
+      <c r="Q54" s="80"/>
+      <c r="R54" s="79"/>
+      <c r="S54" s="80"/>
+      <c r="T54" s="81"/>
     </row>
     <row r="55" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="119"/>
-      <c r="B55" s="120"/>
-      <c r="C55" s="120"/>
-      <c r="D55" s="120"/>
-      <c r="E55" s="121"/>
-      <c r="F55" s="119"/>
-      <c r="G55" s="120"/>
-      <c r="H55" s="194"/>
-      <c r="I55" s="195"/>
-      <c r="J55" s="120"/>
+      <c r="A55" s="83"/>
+      <c r="B55" s="84"/>
+      <c r="C55" s="84"/>
+      <c r="D55" s="84"/>
+      <c r="E55" s="126"/>
+      <c r="F55" s="83"/>
+      <c r="G55" s="84"/>
+      <c r="H55" s="123"/>
+      <c r="I55" s="124"/>
+      <c r="J55" s="84"/>
       <c r="K55" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="L55" s="177"/>
-      <c r="M55" s="177"/>
-      <c r="N55" s="209"/>
-      <c r="O55" s="177"/>
-      <c r="P55" s="205"/>
-      <c r="Q55" s="177"/>
-      <c r="R55" s="205"/>
-      <c r="S55" s="177"/>
-      <c r="T55" s="207"/>
+      <c r="L55" s="80"/>
+      <c r="M55" s="80"/>
+      <c r="N55" s="86"/>
+      <c r="O55" s="80"/>
+      <c r="P55" s="79"/>
+      <c r="Q55" s="80"/>
+      <c r="R55" s="79"/>
+      <c r="S55" s="80"/>
+      <c r="T55" s="82"/>
     </row>
     <row r="56" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="233" t="s">
+      <c r="A56" s="73" t="s">
         <v>67</v>
       </c>
-      <c r="B56" s="233"/>
-      <c r="C56" s="233"/>
-      <c r="D56" s="233"/>
-      <c r="E56" s="233"/>
-      <c r="F56" s="235" t="s">
+      <c r="B56" s="73"/>
+      <c r="C56" s="73"/>
+      <c r="D56" s="73"/>
+      <c r="E56" s="73"/>
+      <c r="F56" s="75" t="s">
         <v>54</v>
       </c>
-      <c r="G56" s="235"/>
-      <c r="H56" s="235"/>
-      <c r="I56" s="235"/>
+      <c r="G56" s="75"/>
+      <c r="H56" s="75"/>
+      <c r="I56" s="75"/>
       <c r="J56" s="30"/>
       <c r="K56" s="43" t="s">
         <v>55</v>
       </c>
-      <c r="L56" s="210"/>
-      <c r="M56" s="211"/>
+      <c r="L56" s="48"/>
+      <c r="M56" s="49"/>
       <c r="N56" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="O56" s="237"/>
-      <c r="P56" s="238"/>
+      <c r="O56" s="77"/>
+      <c r="P56" s="78"/>
       <c r="Q56" s="44" t="s">
         <v>63</v>
       </c>
@@ -5149,28 +5153,28 @@
       <c r="T56" s="47"/>
     </row>
     <row r="57" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="233" t="s">
+      <c r="A57" s="73" t="s">
         <v>68</v>
       </c>
-      <c r="B57" s="233"/>
-      <c r="C57" s="233"/>
-      <c r="D57" s="233"/>
-      <c r="E57" s="234"/>
-      <c r="F57" s="236"/>
-      <c r="G57" s="236"/>
-      <c r="H57" s="236"/>
-      <c r="I57" s="236"/>
+      <c r="B57" s="73"/>
+      <c r="C57" s="73"/>
+      <c r="D57" s="73"/>
+      <c r="E57" s="74"/>
+      <c r="F57" s="76"/>
+      <c r="G57" s="76"/>
+      <c r="H57" s="76"/>
+      <c r="I57" s="76"/>
       <c r="J57" s="30"/>
       <c r="K57" s="43" t="s">
         <v>56</v>
       </c>
-      <c r="L57" s="212"/>
-      <c r="M57" s="212"/>
+      <c r="L57" s="50"/>
+      <c r="M57" s="50"/>
       <c r="N57" s="44" t="s">
         <v>58</v>
       </c>
-      <c r="O57" s="237"/>
-      <c r="P57" s="238"/>
+      <c r="O57" s="77"/>
+      <c r="P57" s="78"/>
       <c r="Q57" s="44" t="s">
         <v>59</v>
       </c>
@@ -5186,10 +5190,10 @@
       <c r="C58" s="33"/>
       <c r="D58" s="33"/>
       <c r="E58" s="33"/>
-      <c r="F58" s="236"/>
-      <c r="G58" s="236"/>
-      <c r="H58" s="236"/>
-      <c r="I58" s="236"/>
+      <c r="F58" s="76"/>
+      <c r="G58" s="76"/>
+      <c r="H58" s="76"/>
+      <c r="I58" s="76"/>
       <c r="J58" s="30"/>
       <c r="K58" s="18"/>
       <c r="L58" s="31"/>
@@ -5203,130 +5207,130 @@
       <c r="T58" s="39"/>
     </row>
     <row r="59" spans="1:20" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="225"/>
-      <c r="B59" s="226"/>
-      <c r="C59" s="226"/>
-      <c r="D59" s="226"/>
-      <c r="E59" s="226"/>
-      <c r="F59" s="226"/>
-      <c r="G59" s="226"/>
-      <c r="H59" s="226"/>
+      <c r="A59" s="65"/>
+      <c r="B59" s="66"/>
+      <c r="C59" s="66"/>
+      <c r="D59" s="66"/>
+      <c r="E59" s="66"/>
+      <c r="F59" s="66"/>
+      <c r="G59" s="66"/>
+      <c r="H59" s="66"/>
       <c r="I59" s="23"/>
-      <c r="K59" s="213" t="s">
+      <c r="K59" s="51" t="s">
         <v>49</v>
       </c>
-      <c r="L59" s="214"/>
-      <c r="M59" s="214"/>
-      <c r="N59" s="214"/>
-      <c r="O59" s="214"/>
-      <c r="P59" s="214"/>
-      <c r="Q59" s="214"/>
-      <c r="R59" s="214"/>
-      <c r="S59" s="214"/>
-      <c r="T59" s="215"/>
+      <c r="L59" s="52"/>
+      <c r="M59" s="52"/>
+      <c r="N59" s="52"/>
+      <c r="O59" s="52"/>
+      <c r="P59" s="52"/>
+      <c r="Q59" s="52"/>
+      <c r="R59" s="52"/>
+      <c r="S59" s="52"/>
+      <c r="T59" s="53"/>
     </row>
     <row r="60" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A60" s="217"/>
-      <c r="B60" s="227" t="s">
+      <c r="A60" s="56"/>
+      <c r="B60" s="67" t="s">
         <v>60</v>
       </c>
-      <c r="C60" s="229" t="s">
+      <c r="C60" s="69" t="s">
         <v>50</v>
       </c>
-      <c r="D60" s="229"/>
-      <c r="E60" s="229"/>
-      <c r="F60" s="229"/>
-      <c r="G60" s="229"/>
-      <c r="H60" s="229"/>
+      <c r="D60" s="69"/>
+      <c r="E60" s="69"/>
+      <c r="F60" s="69"/>
+      <c r="G60" s="69"/>
+      <c r="H60" s="69"/>
       <c r="I60" s="22"/>
-      <c r="K60" s="230" t="s">
+      <c r="K60" s="70" t="s">
         <v>51</v>
       </c>
-      <c r="L60" s="231"/>
-      <c r="M60" s="231"/>
-      <c r="N60" s="231"/>
-      <c r="O60" s="231"/>
-      <c r="P60" s="231"/>
-      <c r="Q60" s="231"/>
-      <c r="R60" s="231"/>
-      <c r="S60" s="231"/>
-      <c r="T60" s="232"/>
+      <c r="L60" s="71"/>
+      <c r="M60" s="71"/>
+      <c r="N60" s="71"/>
+      <c r="O60" s="71"/>
+      <c r="P60" s="71"/>
+      <c r="Q60" s="71"/>
+      <c r="R60" s="71"/>
+      <c r="S60" s="71"/>
+      <c r="T60" s="72"/>
     </row>
     <row r="61" spans="1:20" ht="39.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="217"/>
-      <c r="B61" s="228"/>
-      <c r="C61" s="229"/>
-      <c r="D61" s="229"/>
-      <c r="E61" s="229"/>
-      <c r="F61" s="229"/>
-      <c r="G61" s="229"/>
-      <c r="H61" s="229"/>
+      <c r="A61" s="56"/>
+      <c r="B61" s="68"/>
+      <c r="C61" s="69"/>
+      <c r="D61" s="69"/>
+      <c r="E61" s="69"/>
+      <c r="F61" s="69"/>
+      <c r="G61" s="69"/>
+      <c r="H61" s="69"/>
       <c r="I61" s="22"/>
-      <c r="K61" s="230"/>
-      <c r="L61" s="231"/>
-      <c r="M61" s="231"/>
-      <c r="N61" s="231"/>
-      <c r="O61" s="231"/>
-      <c r="P61" s="231"/>
-      <c r="Q61" s="231"/>
-      <c r="R61" s="231"/>
-      <c r="S61" s="231"/>
-      <c r="T61" s="232"/>
+      <c r="K61" s="70"/>
+      <c r="L61" s="71"/>
+      <c r="M61" s="71"/>
+      <c r="N61" s="71"/>
+      <c r="O61" s="71"/>
+      <c r="P61" s="71"/>
+      <c r="Q61" s="71"/>
+      <c r="R61" s="71"/>
+      <c r="S61" s="71"/>
+      <c r="T61" s="72"/>
     </row>
     <row r="62" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="156"/>
-      <c r="B62" s="216"/>
-      <c r="C62" s="216"/>
-      <c r="D62" s="216"/>
-      <c r="E62" s="216"/>
-      <c r="F62" s="216"/>
-      <c r="G62" s="216"/>
-      <c r="H62" s="216"/>
+      <c r="A62" s="54"/>
+      <c r="B62" s="55"/>
+      <c r="C62" s="55"/>
+      <c r="D62" s="55"/>
+      <c r="E62" s="55"/>
+      <c r="F62" s="55"/>
+      <c r="G62" s="55"/>
+      <c r="H62" s="55"/>
       <c r="I62" s="22"/>
       <c r="K62" s="24"/>
-      <c r="L62" s="220"/>
-      <c r="M62" s="220"/>
-      <c r="N62" s="220"/>
-      <c r="O62" s="220"/>
-      <c r="P62" s="220"/>
-      <c r="Q62" s="220"/>
-      <c r="S62" s="221"/>
-      <c r="T62" s="222"/>
+      <c r="L62" s="59"/>
+      <c r="M62" s="59"/>
+      <c r="N62" s="59"/>
+      <c r="O62" s="59"/>
+      <c r="P62" s="59"/>
+      <c r="Q62" s="59"/>
+      <c r="S62" s="61"/>
+      <c r="T62" s="62"/>
     </row>
     <row r="63" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A63" s="217"/>
-      <c r="B63" s="216"/>
-      <c r="C63" s="216"/>
-      <c r="D63" s="216"/>
-      <c r="E63" s="216"/>
-      <c r="F63" s="216"/>
-      <c r="G63" s="216"/>
-      <c r="H63" s="216"/>
+      <c r="A63" s="56"/>
+      <c r="B63" s="55"/>
+      <c r="C63" s="55"/>
+      <c r="D63" s="55"/>
+      <c r="E63" s="55"/>
+      <c r="F63" s="55"/>
+      <c r="G63" s="55"/>
+      <c r="H63" s="55"/>
       <c r="I63" s="22"/>
       <c r="K63" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="L63" s="85"/>
-      <c r="M63" s="85"/>
-      <c r="N63" s="85"/>
-      <c r="O63" s="85"/>
-      <c r="P63" s="85"/>
-      <c r="Q63" s="85"/>
+      <c r="L63" s="60"/>
+      <c r="M63" s="60"/>
+      <c r="N63" s="60"/>
+      <c r="O63" s="60"/>
+      <c r="P63" s="60"/>
+      <c r="Q63" s="60"/>
       <c r="R63" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="S63" s="223"/>
-      <c r="T63" s="224"/>
+      <c r="S63" s="63"/>
+      <c r="T63" s="64"/>
     </row>
     <row r="64" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A64" s="218"/>
-      <c r="B64" s="219"/>
-      <c r="C64" s="219"/>
-      <c r="D64" s="219"/>
-      <c r="E64" s="219"/>
-      <c r="F64" s="219"/>
-      <c r="G64" s="219"/>
-      <c r="H64" s="219"/>
+      <c r="A64" s="57"/>
+      <c r="B64" s="58"/>
+      <c r="C64" s="58"/>
+      <c r="D64" s="58"/>
+      <c r="E64" s="58"/>
+      <c r="F64" s="58"/>
+      <c r="G64" s="58"/>
+      <c r="H64" s="58"/>
       <c r="I64" s="26"/>
       <c r="J64" s="4"/>
       <c r="K64" s="27"/>
@@ -5342,45 +5346,156 @@
     </row>
   </sheetData>
   <mergeCells count="213">
-    <mergeCell ref="L56:M56"/>
-    <mergeCell ref="L57:M57"/>
-    <mergeCell ref="K59:T59"/>
-    <mergeCell ref="A62:H64"/>
-    <mergeCell ref="L62:Q63"/>
-    <mergeCell ref="S62:T63"/>
-    <mergeCell ref="A59:A61"/>
-    <mergeCell ref="B59:H59"/>
-    <mergeCell ref="B60:B61"/>
-    <mergeCell ref="C60:H61"/>
-    <mergeCell ref="K60:T61"/>
-    <mergeCell ref="A56:E56"/>
-    <mergeCell ref="A57:E57"/>
-    <mergeCell ref="F56:I56"/>
-    <mergeCell ref="F57:I58"/>
-    <mergeCell ref="O56:P56"/>
-    <mergeCell ref="O57:P57"/>
-    <mergeCell ref="R54:R55"/>
-    <mergeCell ref="S54:S55"/>
-    <mergeCell ref="T54:T55"/>
-    <mergeCell ref="A55:B55"/>
-    <mergeCell ref="N54:N55"/>
-    <mergeCell ref="O54:O55"/>
-    <mergeCell ref="P54:P55"/>
-    <mergeCell ref="Q54:Q55"/>
-    <mergeCell ref="L54:M55"/>
-    <mergeCell ref="O52:O53"/>
-    <mergeCell ref="O50:O51"/>
-    <mergeCell ref="L52:M53"/>
-    <mergeCell ref="P52:P53"/>
-    <mergeCell ref="Q52:Q53"/>
-    <mergeCell ref="R52:R53"/>
-    <mergeCell ref="S52:S53"/>
-    <mergeCell ref="T52:T53"/>
-    <mergeCell ref="Q50:Q51"/>
-    <mergeCell ref="R50:R51"/>
-    <mergeCell ref="S50:S51"/>
-    <mergeCell ref="T50:T51"/>
-    <mergeCell ref="P50:P51"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="F44:I44"/>
+    <mergeCell ref="F45:I45"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="F37:I37"/>
+    <mergeCell ref="F36:I36"/>
+    <mergeCell ref="F40:I40"/>
+    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="F38:I38"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="P3:T4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:F6"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="H1:L4"/>
+    <mergeCell ref="M1:M2"/>
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="O1:T2"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:G4"/>
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="N3:N4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:I7"/>
+    <mergeCell ref="J5:J7"/>
+    <mergeCell ref="K5:Q7"/>
+    <mergeCell ref="R5:R7"/>
+    <mergeCell ref="T5:T7"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="A11:B12"/>
+    <mergeCell ref="C11:E12"/>
+    <mergeCell ref="F11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="K11:L12"/>
+    <mergeCell ref="M11:T12"/>
+    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="K8:Q10"/>
+    <mergeCell ref="R8:R10"/>
+    <mergeCell ref="T8:T10"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="B7:F8"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="I8:I10"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="Q13:R14"/>
+    <mergeCell ref="S13:T14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="J15:J49"/>
+    <mergeCell ref="A13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:E14"/>
+    <mergeCell ref="F13:I14"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="K13:K14"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="M13:N14"/>
+    <mergeCell ref="O13:P14"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:I22"/>
+    <mergeCell ref="F30:I30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="F46:I46"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:I31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F32:I32"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="F33:I33"/>
+    <mergeCell ref="F34:I34"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="F41:I41"/>
+    <mergeCell ref="F42:I42"/>
+    <mergeCell ref="F43:I43"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:I27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="A29:B29"/>
     <mergeCell ref="K52:K53"/>
     <mergeCell ref="N52:N53"/>
     <mergeCell ref="K50:K51"/>
@@ -5405,156 +5520,45 @@
     <mergeCell ref="F48:I48"/>
     <mergeCell ref="A48:B48"/>
     <mergeCell ref="D48:E48"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:I27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="F30:I30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="F46:I46"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:I31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:I32"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="F24:I24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="F21:I21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:I22"/>
-    <mergeCell ref="F20:I20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="M13:N14"/>
-    <mergeCell ref="O13:P14"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="Q13:R14"/>
-    <mergeCell ref="S13:T14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="J15:J49"/>
-    <mergeCell ref="A13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:E14"/>
-    <mergeCell ref="F13:I14"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="K13:K14"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:I23"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A11:B12"/>
-    <mergeCell ref="C11:E12"/>
-    <mergeCell ref="F11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="K11:L12"/>
-    <mergeCell ref="M11:T12"/>
-    <mergeCell ref="J8:J10"/>
-    <mergeCell ref="K8:Q10"/>
-    <mergeCell ref="R8:R10"/>
-    <mergeCell ref="T8:T10"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="B7:F8"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="I8:I10"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="P3:T4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:F6"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="H1:L4"/>
-    <mergeCell ref="M1:M2"/>
-    <mergeCell ref="N1:N2"/>
-    <mergeCell ref="O1:T2"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:G4"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="N3:N4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I5:I7"/>
-    <mergeCell ref="J5:J7"/>
-    <mergeCell ref="K5:Q7"/>
-    <mergeCell ref="R5:R7"/>
-    <mergeCell ref="T5:T7"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="F33:I33"/>
-    <mergeCell ref="F34:I34"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="F41:I41"/>
-    <mergeCell ref="F42:I42"/>
-    <mergeCell ref="F43:I43"/>
-    <mergeCell ref="F44:I44"/>
-    <mergeCell ref="F45:I45"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="F37:I37"/>
-    <mergeCell ref="F36:I36"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="F40:I40"/>
-    <mergeCell ref="F39:I39"/>
-    <mergeCell ref="F38:I38"/>
+    <mergeCell ref="O52:O53"/>
+    <mergeCell ref="O50:O51"/>
+    <mergeCell ref="L52:M53"/>
+    <mergeCell ref="P52:P53"/>
+    <mergeCell ref="Q52:Q53"/>
+    <mergeCell ref="R52:R53"/>
+    <mergeCell ref="S52:S53"/>
+    <mergeCell ref="T52:T53"/>
+    <mergeCell ref="Q50:Q51"/>
+    <mergeCell ref="R50:R51"/>
+    <mergeCell ref="S50:S51"/>
+    <mergeCell ref="T50:T51"/>
+    <mergeCell ref="P50:P51"/>
+    <mergeCell ref="R54:R55"/>
+    <mergeCell ref="S54:S55"/>
+    <mergeCell ref="T54:T55"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="N54:N55"/>
+    <mergeCell ref="O54:O55"/>
+    <mergeCell ref="P54:P55"/>
+    <mergeCell ref="Q54:Q55"/>
+    <mergeCell ref="L54:M55"/>
+    <mergeCell ref="L56:M56"/>
+    <mergeCell ref="L57:M57"/>
+    <mergeCell ref="K59:T59"/>
+    <mergeCell ref="A62:H64"/>
+    <mergeCell ref="L62:Q63"/>
+    <mergeCell ref="S62:T63"/>
+    <mergeCell ref="A59:A61"/>
+    <mergeCell ref="B59:H59"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="C60:H61"/>
+    <mergeCell ref="K60:T61"/>
+    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="F56:I56"/>
+    <mergeCell ref="F57:I58"/>
+    <mergeCell ref="O56:P56"/>
+    <mergeCell ref="O57:P57"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="37" orientation="landscape" r:id="rId1"/>
@@ -5636,6 +5640,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="168aac3c-b196-482c-82c2-e21ec3905f91" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010012E1092C228E9843AE24A7AB177EE014" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5d1156d0328de5d9cb25b668e7661c3f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="62c34b96-1298-4448-bbb4-05585e6704b5" xmlns:ns4="168aac3c-b196-482c-82c2-e21ec3905f91" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ce5195017d4bfad0a0e1097928d06013" ns3:_="" ns4:_="">
     <xsd:import namespace="62c34b96-1298-4448-bbb4-05585e6704b5"/>
@@ -5862,38 +5883,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="168aac3c-b196-482c-82c2-e21ec3905f91" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A70B0A65-1B60-4D8E-A9DC-845EE84FC104}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{917DF9EF-3853-4349-A9A5-379671540C73}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="62c34b96-1298-4448-bbb4-05585e6704b5"/>
-    <ds:schemaRef ds:uri="168aac3c-b196-482c-82c2-e21ec3905f91"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5916,9 +5909,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{917DF9EF-3853-4349-A9A5-379671540C73}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A70B0A65-1B60-4D8E-A9DC-845EE84FC104}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="62c34b96-1298-4448-bbb4-05585e6704b5"/>
+    <ds:schemaRef ds:uri="168aac3c-b196-482c-82c2-e21ec3905f91"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>